<commit_message>
added a talk: kek
</commit_message>
<xml_diff>
--- a/talklists/talklist.xlsx
+++ b/talklists/talklist.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sugiyamasunao/Documents/appforms/cv/talklists/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sugiyamasunao/Documents/writing/cv/talklists/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F6B43C7-B39E-1A40-84EB-09609667B43C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{505ED053-D816-9142-853D-3EEEDDA05D8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="220">
   <si>
     <t>title</t>
   </si>
@@ -876,6 +876,18 @@
   </si>
   <si>
     <t>https://www.asiaa.sinica.edu.tw/activity/colloquium.php</t>
+  </si>
+  <si>
+    <t>https://cosmophysics.gitlab.io/jointseminar.gitlab.io/sugiyama20260615.html</t>
+  </si>
+  <si>
+    <t>Probing Primordial Black Hole Dark Matter with Subaru HSC Microlensing Observations of M31</t>
+  </si>
+  <si>
+    <t>IPNS Joint Experimental-Theoretica Cosmology Seminar</t>
+  </si>
+  <si>
+    <t>Yuji Chinone</t>
   </si>
 </sst>
 </file>
@@ -3795,7 +3807,7 @@
       <c r="M38" s="8">
         <v>1</v>
       </c>
-      <c r="N38" s="16" t="s">
+      <c r="N38" s="38" t="s">
         <v>153</v>
       </c>
       <c r="O38" s="19" t="s">
@@ -4146,6 +4158,9 @@
       <c r="K48" s="57">
         <v>1</v>
       </c>
+      <c r="M48" s="40">
+        <v>1</v>
+      </c>
       <c r="N48" s="61" t="s">
         <v>207</v>
       </c>
@@ -4178,6 +4193,9 @@
       <c r="K49" s="47">
         <v>1</v>
       </c>
+      <c r="M49" s="1">
+        <v>1</v>
+      </c>
       <c r="N49" s="62" t="s">
         <v>214</v>
       </c>
@@ -4208,6 +4226,41 @@
         <v>1</v>
       </c>
       <c r="K50" s="40">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:18" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="49" t="s">
+        <v>217</v>
+      </c>
+      <c r="C51" s="47">
+        <v>2026</v>
+      </c>
+      <c r="D51" s="47">
+        <v>6</v>
+      </c>
+      <c r="E51" s="41" t="s">
+        <v>69</v>
+      </c>
+      <c r="F51" s="41" t="s">
+        <v>218</v>
+      </c>
+      <c r="I51" s="1">
+        <v>1</v>
+      </c>
+      <c r="K51" s="47">
+        <v>1</v>
+      </c>
+      <c r="M51" s="1">
+        <v>1</v>
+      </c>
+      <c r="N51" s="33" t="s">
+        <v>219</v>
+      </c>
+      <c r="O51" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="R51" s="33">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added a talk at PPP 2026 08 27
</commit_message>
<xml_diff>
--- a/talklists/talklist.xlsx
+++ b/talklists/talklist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sugiyamasunao/Documents/writing/cv/talklists/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{493EE602-5EF2-D94B-BA75-169598A7A210}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AE69A62-EA3A-444E-977A-364E38C176C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="228">
   <si>
     <t>title</t>
   </si>
@@ -894,6 +894,24 @@
   </si>
   <si>
     <t>https://roman-hlis-cosmology.caltech.edu/news/2024-f2f</t>
+  </si>
+  <si>
+    <t>Observational exploration of primordial black holes</t>
+  </si>
+  <si>
+    <t>YITP</t>
+  </si>
+  <si>
+    <t>Progress in Partcles Physics</t>
+  </si>
+  <si>
+    <t>Kodai Sakurai</t>
+  </si>
+  <si>
+    <t>https://indico.yukawa.kyoto-u.ac.jp/event/95/overview</t>
+  </si>
+  <si>
+    <t>原始ブラックホールの観測的探査</t>
   </si>
 </sst>
 </file>
@@ -4276,7 +4294,45 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:18" s="40" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="52" spans="1:18" s="40" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A52" s="61" t="s">
+        <v>227</v>
+      </c>
+      <c r="B52" s="61" t="s">
+        <v>222</v>
+      </c>
+      <c r="C52" s="40">
+        <v>2026</v>
+      </c>
+      <c r="D52" s="40">
+        <v>8</v>
+      </c>
+      <c r="E52" s="61" t="s">
+        <v>223</v>
+      </c>
+      <c r="F52" s="61" t="s">
+        <v>224</v>
+      </c>
+      <c r="H52" s="40">
+        <v>1</v>
+      </c>
+      <c r="K52" s="40">
+        <v>1</v>
+      </c>
+      <c r="M52" s="40">
+        <v>1</v>
+      </c>
+      <c r="N52" s="61" t="s">
+        <v>225</v>
+      </c>
+      <c r="O52" s="58" t="s">
+        <v>226</v>
+      </c>
+      <c r="Q52" s="61"/>
+      <c r="R52" s="40">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="O2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
@@ -4315,6 +4371,7 @@
     <hyperlink ref="O49" r:id="rId34" xr:uid="{7FA0972F-0B7F-834A-A6FD-87E313E18CDA}"/>
     <hyperlink ref="O45" r:id="rId35" xr:uid="{2352478C-31CE-D648-B159-05F52D2D7F99}"/>
     <hyperlink ref="O46" r:id="rId36" xr:uid="{27B9BA78-A76E-4544-BD20-2EA63281B52A}"/>
+    <hyperlink ref="O52" r:id="rId37" xr:uid="{4C59414C-6EB5-6641-B099-AE6C98E8A444}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>

</xml_diff>